<commit_message>
Locate unregistered outputs and bind native evidence to its corpus - carry the output name and sha-256 on registration failures through a shared recovery exception, filesystem, sharepoint and tools - fail the native record unless results match the exact manifest, case ids, output hashes, every check and the controls - keep corpus json and markdown as lf text so the manifest hash is stable and git diff --check passes - rerun office on the regenerated corpus, 70 of 70 cases, and prove the fixes with 12 removal probes
</commit_message>
<xml_diff>
--- a/tests/OfficeAgent.Tests/Corpus/v1.0.0/native/inputs/x-appendtablerows.xlsx
+++ b/tests/OfficeAgent.Tests/Corpus/v1.0.0/native/inputs/x-appendtablerows.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="7" r:id="Rbeb5732cf0fa4649"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="7" r:id="Rfb25d51505b84c28"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -81,7 +81,7 @@
     </x:row>
   </x:sheetData>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03302f104fe6457c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b29c2afcfd34aaa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add formula calculation, Word conformance verbs and core properties for 1.2.0
- add optional OfficeAgent.Excel.Calculation with an allowlisted ClosedXML engine, per-connection settings and formula-error rejection
- add the link and mergeTableCells verbs, numberingId on format, list nodes, compatibility mode and FindHit.ParaId
- store post-2007 Excel functions with their _xlfn. prefix so setCell formulas no longer show #NAME? in Excel
- republish the native Office record with opened controls and new cases, and ship the tenth package in release checks
</commit_message>
<xml_diff>
--- a/tests/OfficeAgent.Tests/Corpus/v1.0.0/native/inputs/x-appendtablerows.xlsx
+++ b/tests/OfficeAgent.Tests/Corpus/v1.0.0/native/inputs/x-appendtablerows.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="7" r:id="Rfb25d51505b84c28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="7" r:id="R17c4b5a2ea7a4df7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -81,7 +81,7 @@
     </x:row>
   </x:sheetData>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b29c2afcfd34aaa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff1c5024fba44bf9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add report refresh, formatting-safe translation and multi-document edits
- refresh word reports and powerpoint decks from an excel workbook through xl: bindings with refresh_document
- add fillTable, setChartData and bindData verbs plus formatted cell values and defined names in excel inspection
- keep inline formatting when rewriting a paragraph through markedText and withMarked
- apply one plan to many documents with edit_documents and match every occurrence with "match": "all"
</commit_message>
<xml_diff>
--- a/tests/OfficeAgent.Tests/Corpus/v1.0.0/native/inputs/x-appendtablerows.xlsx
+++ b/tests/OfficeAgent.Tests/Corpus/v1.0.0/native/inputs/x-appendtablerows.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="7" r:id="R17c4b5a2ea7a4df7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="7" r:id="R8d508d72d97a42b0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -81,7 +81,7 @@
     </x:row>
   </x:sheetData>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff1c5024fba44bf9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1b0934e5d5c4fe2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix the review findings in refresh, table fills and marked rewrites
- refuse a marked rewrite of a paragraph holding tabs, breaks, fields, note references or pictures
- keep comment and bookmark anchors in filled word cells and strip them from copied rows
- format accounting and currency built-ins, drop copied slide row ids, and guard combination charts
- read each workbook sheet once per refresh and keep bound officeagent charts updatable
</commit_message>
<xml_diff>
--- a/tests/OfficeAgent.Tests/Corpus/v1.0.0/native/inputs/x-appendtablerows.xlsx
+++ b/tests/OfficeAgent.Tests/Corpus/v1.0.0/native/inputs/x-appendtablerows.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="7" r:id="R8d508d72d97a42b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="7" r:id="R8f2ae60a883b4d1d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -81,7 +81,7 @@
     </x:row>
   </x:sheetData>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1b0934e5d5c4fe2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0ac6fe1bded429b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Put new slides on a template's own layouts by name
- resolve insertSlide layouts against the names powerpoint shows, qualified by master when they repeat
- give a slide on a named layout every placeholder the layout defines, under its own shape names
- list each deck's layouts and placeholders in inspect_document and refuse text a layout has no place for
- republish the native record at 84 of 84 cases with a named-layout slide case
</commit_message>
<xml_diff>
--- a/tests/OfficeAgent.Tests/Corpus/v1.0.0/native/inputs/x-appendtablerows.xlsx
+++ b/tests/OfficeAgent.Tests/Corpus/v1.0.0/native/inputs/x-appendtablerows.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="7" r:id="R8f2ae60a883b4d1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="7" r:id="R3e1121b643084885"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -81,7 +81,7 @@
     </x:row>
   </x:sheetData>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0ac6fe1bded429b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc524914ed2e47b5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>